<commit_message>
TW-link toevoegen en functies in het werkboek aanklikbaar maken
- TW-functie toegevoegd aan de links van de financiële les
- BET, HW, RENTE en TW op blad 1 van het startbestand linken nu naar
  hun Google Help-pagina, zoals in de originele oefening

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wu5SnViXCqMtBpPMNxsmhA
</commit_message>
<xml_diff>
--- a/bestanden/werkbladen-oefeningen-START.xlsx
+++ b/bestanden/werkbladen-oefeningen-START.xlsx
@@ -106,7 +106,7 @@
     <t xml:space="preserve">Wat als ik maandelijks afbetaal in plaats van jaarlijks? (let op de periodes)</t>
   </si>
   <si>
-    <t xml:space="preserve">Functies die je hier kunt gebruiken</t>
+    <t xml:space="preserve">Functies die je hier kunt gebruiken (klik voor de uitleg)</t>
   </si>
   <si>
     <t xml:space="preserve">BET</t>
@@ -425,7 +425,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="&quot;€ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -482,6 +482,15 @@
       <i val="true"/>
       <sz val="11"/>
       <color rgb="FF7A8699"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -582,24 +591,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -607,51 +620,51 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -667,15 +680,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -683,11 +700,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -724,7 +741,7 @@
       <rgbColor rgb="FFDCE6F5"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF0563C1"/>
       <rgbColor rgb="FFBDD7EE"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -946,112 +963,112 @@
   <dimension ref="A1:E19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="B3" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="6" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4"/>
+      <c r="B12" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7"/>
-      <c r="B13" s="6" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8"/>
+      <c r="B13" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8"/>
-      <c r="B14" s="6" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9"/>
+      <c r="B14" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1077,172 +1094,172 @@
   <dimension ref="A1:D27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="12" t="n">
         <v>16000</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="13" t="n">
         <v>0.03</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="13"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="B10" s="14"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="14" t="n">
+      <c r="B11" s="15" t="n">
         <v>-200</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="15"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+      <c r="B12" s="16"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="B13" s="17"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="15"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
+      <c r="B16" s="16"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="15"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+      <c r="B17" s="16"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="15"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="B18" s="16"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18"/>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="19"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1255,6 +1272,12 @@
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="A26:D27"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A21" r:id="rId1" display="BET"/>
+    <hyperlink ref="A22" r:id="rId2" display="HW"/>
+    <hyperlink ref="A23" r:id="rId3" display="RENTE"/>
+    <hyperlink ref="A24" r:id="rId4" display="TW"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1273,106 +1296,106 @@
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="15" t="n">
         <v>-200</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="13" t="n">
         <v>0.02</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="15"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="B9" s="16"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="15"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="B10" s="16"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="15"/>
+      <c r="B11" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1399,241 +1422,241 @@
   <dimension ref="A1:F26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="22" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="22" t="str">
+      <c r="B7" s="23" t="str">
         <f aca="false">IFERROR(VLOOKUP($A7,Gegevens!$A$5:$C$18,2,FALSE()),"niet gevonden")</f>
         <v>Processor 6 cores, 4,1 GHz</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="24" t="n">
         <f aca="false">IFERROR(VLOOKUP($A7,Gegevens!$A$5:$C$18,3,FALSE()),0)</f>
         <v>189</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="24" t="n">
         <f aca="false">C7*D7</f>
         <v>189</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="10" t="n">
+      <c r="B8" s="4"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="15"/>
-      <c r="F8" s="10"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="E8" s="16"/>
+      <c r="F8" s="11"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="10" t="n">
+      <c r="B9" s="4"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="15"/>
-      <c r="F9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="E9" s="16"/>
+      <c r="F9" s="11"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="10" t="n">
+      <c r="B10" s="4"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="15"/>
-      <c r="F10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="E10" s="16"/>
+      <c r="F10" s="11"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="10" t="n">
+      <c r="B11" s="4"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="15"/>
-      <c r="F11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+      <c r="E11" s="16"/>
+      <c r="F11" s="11"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="10" t="n">
+      <c r="B12" s="4"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="15"/>
-      <c r="F12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+      <c r="E12" s="16"/>
+      <c r="F12" s="11"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="10" t="n">
+      <c r="B13" s="4"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="15"/>
-      <c r="F13" s="10"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+      <c r="E13" s="16"/>
+      <c r="F13" s="11"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="10" t="n">
+      <c r="B14" s="4"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="15"/>
-      <c r="F14" s="22" t="s">
+      <c r="E14" s="16"/>
+      <c r="F14" s="23" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D16" s="17" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D16" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="15"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D17" s="17" t="s">
+      <c r="E16" s="16"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D17" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D18" s="17" t="s">
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D18" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="E18" s="15"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D19" s="17" t="s">
+      <c r="E18" s="16"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D19" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="E19" s="15"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="E19" s="16"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1659,116 +1682,116 @@
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="22" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="15"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="C7" s="16"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="10" t="str">
+      <c r="B8" s="11" t="str">
         <f aca="false">B7</f>
         <v>Q3</v>
       </c>
-      <c r="C8" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="C8" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="C10" s="15"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="C10" s="16"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="C11" s="15"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+      <c r="C11" s="16"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="C12" s="15"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="C12" s="16"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1794,149 +1817,149 @@
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B8" s="3"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="B8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="15"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="B9" s="16"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
+      <c r="B10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="D18" s="22" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="14" t="n">
+      <c r="B19" s="27"/>
+      <c r="C19" s="15" t="n">
         <v>948</v>
       </c>
-      <c r="D19" s="15"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="n">
+      <c r="D19" s="16"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="n">
         <v>34</v>
       </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="14" t="n">
+      <c r="B20" s="27"/>
+      <c r="C20" s="15" t="n">
         <v>2686</v>
       </c>
-      <c r="D20" s="15"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="n">
+      <c r="D20" s="16"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="n">
         <v>73</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="14" t="n">
+      <c r="B21" s="27"/>
+      <c r="C21" s="15" t="n">
         <v>5767</v>
       </c>
-      <c r="D21" s="15"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="n">
+      <c r="D21" s="16"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="14" t="n">
+      <c r="B22" s="27"/>
+      <c r="C22" s="15" t="n">
         <v>11850</v>
       </c>
-      <c r="D22" s="15"/>
+      <c r="D22" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1963,294 +1986,294 @@
   <dimension ref="A1:I24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="22" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" s="15" t="n">
         <v>79</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="13" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="15" t="n">
         <v>189</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="13" t="n">
         <v>0.03</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="15" t="n">
         <v>329</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="13" t="n">
         <v>0.07</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="15" t="n">
         <v>549</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="13" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="15" t="n">
         <v>279</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="13" t="n">
         <v>0.18</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="15" t="n">
         <v>489</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="15" t="n">
         <v>899</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="E11" s="28" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <v>94.5</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="15" t="n">
         <v>109</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="15" t="n">
         <v>179</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="15" t="n">
         <v>89</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="C16" s="14" t="n">
+      <c r="C16" s="15" t="n">
         <v>64</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="C17" s="15" t="n">
         <v>79</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C18" s="15" t="n">
         <v>139</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="25" t="s">
         <v>124</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="25" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B23" s="12" t="n">
         <v>612</v>
       </c>
-      <c r="C23" s="11" t="n">
+      <c r="C23" s="12" t="n">
         <v>548</v>
       </c>
-      <c r="D23" s="11" t="n">
+      <c r="D23" s="12" t="n">
         <v>497</v>
       </c>
-      <c r="E23" s="11" t="n">
+      <c r="E23" s="12" t="n">
         <v>579</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="B24" s="10" t="n">
+      <c r="B24" s="11" t="n">
         <v>184</v>
       </c>
-      <c r="C24" s="10" t="n">
+      <c r="C24" s="11" t="n">
         <v>236</v>
       </c>
-      <c r="D24" s="10" t="n">
+      <c r="D24" s="11" t="n">
         <v>311</v>
       </c>
-      <c r="E24" s="10" t="n">
+      <c r="E24" s="11" t="n">
         <v>402</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Sheets-materiaal nagelezen en gecorrigeerd
- waarschuwingskop staat nu per opdracht; de werkbladbundel werd ten
  onrechte "met opzet verknoeid" genoemd
- financiële bedragen exact gemaakt: HW 10.991, TW 13.272, rente 1.468
  (ook in het leningschema en de bijhorende vraag)
- wb07: "=SOM(B2+B3)" is een geldige formule en kon geen afleider zijn
- fi01: tip verklapte het antwoord
- zo10: bereik zonder dollartekens, terwijl de fiches er net op hameren
- zo22: antwoord en uitleg noemden een ander aantal gewoontes
- uitleg over puntkomma versus komma (landinstelling) in fiche W5 en in
  het startbestand

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wu5SnViXCqMtBpPMNxsmhA
</commit_message>
<xml_diff>
--- a/bestanden/werkbladen-oefeningen-START.xlsx
+++ b/bestanden/werkbladen-oefeningen-START.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="130">
   <si>
     <t xml:space="preserve">Werkbladen — oefeningenbundel</t>
   </si>
@@ -62,6 +62,12 @@
   </si>
   <si>
     <t xml:space="preserve">Op de cursuspagina's Werkbladen (basis, financieel en zoeken) staat alles wat je hier nodig hebt, met schema's en fiches.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puntkomma of komma?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In deze bundel scheiden we de argumenten van een functie met een puntkomma, bv. =SOM(B2;B3). Typt jouw Sheets liever een komma, dan staat de regio anders ingesteld: Bestand → Instellingen → Landinstelling. Allebei is goed, als je maar consequent bent met wat jouw bestand verwacht.</t>
   </si>
   <si>
     <t xml:space="preserve">Oefening 1 — Een lening voor een nieuwe wagen</t>
@@ -425,7 +431,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="&quot;€ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -482,6 +488,19 @@
       <i val="true"/>
       <sz val="11"/>
       <color rgb="FF7A8699"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -591,7 +610,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -636,6 +655,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -664,7 +691,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -704,7 +731,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -960,7 +987,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
@@ -1070,11 +1097,40 @@
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
     </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A6:E9"/>
     <mergeCell ref="A18:E19"/>
+    <mergeCell ref="A21:E23"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1101,7 +1157,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1109,7 +1165,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1117,7 +1173,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1130,136 +1186,136 @@
       <c r="D5" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="12" t="n">
+      <c r="A7" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="14" t="n">
         <v>16000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="13" t="n">
+      <c r="A8" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="15" t="n">
         <v>0.03</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="11" t="n">
+      <c r="A9" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="13" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="14"/>
+      <c r="A10" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="15" t="n">
+      <c r="A11" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="17" t="n">
         <v>-200</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="16"/>
+      <c r="A12" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="17"/>
+      <c r="A13" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="19"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="16"/>
+      <c r="A16" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="18"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="16"/>
+      <c r="A17" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="18"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="16"/>
+      <c r="A18" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
+      <c r="A21" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
+      <c r="A22" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
+      <c r="A23" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
+      <c r="A24" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
+      <c r="A26" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19"/>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
+      <c r="A27" s="21"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1303,7 +1359,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1311,7 +1367,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1324,78 +1380,78 @@
       <c r="D4" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="15" t="n">
+      <c r="A6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="17" t="n">
         <v>-200</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="13" t="n">
+      <c r="A7" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="15" t="n">
         <v>0.02</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="11" t="n">
+      <c r="A8" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="13" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="16"/>
+      <c r="A9" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" s="16"/>
+      <c r="A10" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="16"/>
+      <c r="A11" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
+      <c r="A13" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
+      <c r="A15" s="23"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
+      <c r="A16" s="23"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
+      <c r="A17" s="23"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1432,7 +1488,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1442,7 +1498,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1459,166 +1515,166 @@
       <c r="F4" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" s="22" t="s">
+      <c r="A6" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="B6" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="C6" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="D6" s="24" t="s">
         <v>52</v>
       </c>
+      <c r="E6" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="24" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" s="23" t="str">
+      <c r="A7" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="25" t="str">
         <f aca="false">IFERROR(VLOOKUP($A7,Gegevens!$A$5:$C$18,2,FALSE()),"niet gevonden")</f>
         <v>Processor 6 cores, 4,1 GHz</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="26" t="n">
         <f aca="false">IFERROR(VLOOKUP($A7,Gegevens!$A$5:$C$18,3,FALSE()),0)</f>
         <v>189</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="26" t="n">
         <f aca="false">C7*D7</f>
         <v>189</v>
       </c>
-      <c r="F7" s="23" t="s">
-        <v>54</v>
+      <c r="F7" s="25" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>55</v>
+      <c r="A8" s="13" t="s">
+        <v>57</v>
       </c>
       <c r="B8" s="4"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="11" t="n">
+      <c r="C8" s="18"/>
+      <c r="D8" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="16"/>
-      <c r="F8" s="11"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>56</v>
+      <c r="A9" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="B9" s="4"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="11" t="n">
+      <c r="C9" s="18"/>
+      <c r="D9" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="16"/>
-      <c r="F9" s="11"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>57</v>
+      <c r="A10" s="13" t="s">
+        <v>59</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="11" t="n">
+      <c r="C10" s="18"/>
+      <c r="D10" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="11"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>58</v>
+      <c r="A11" s="13" t="s">
+        <v>60</v>
       </c>
       <c r="B11" s="4"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="11" t="n">
+      <c r="C11" s="18"/>
+      <c r="D11" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="16"/>
-      <c r="F11" s="11"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>59</v>
+      <c r="A12" s="13" t="s">
+        <v>61</v>
       </c>
       <c r="B12" s="4"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="11" t="n">
+      <c r="C12" s="18"/>
+      <c r="D12" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="16"/>
-      <c r="F12" s="11"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>60</v>
+      <c r="A13" s="13" t="s">
+        <v>62</v>
       </c>
       <c r="B13" s="4"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="11" t="n">
+      <c r="C13" s="18"/>
+      <c r="D13" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="16"/>
-      <c r="F13" s="11"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="13"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>61</v>
+      <c r="A14" s="13" t="s">
+        <v>63</v>
       </c>
       <c r="B14" s="4"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="11" t="n">
+      <c r="C14" s="18"/>
+      <c r="D14" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="23" t="s">
-        <v>62</v>
+      <c r="E14" s="18"/>
+      <c r="F14" s="25" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D16" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="E16" s="16"/>
+      <c r="D16" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" s="18"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D17" s="25" t="s">
-        <v>64</v>
+      <c r="D17" s="27" t="s">
+        <v>66</v>
       </c>
       <c r="E17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D18" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="E18" s="16"/>
+      <c r="D18" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D19" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="E19" s="16"/>
+      <c r="D19" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1688,7 +1744,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1698,7 +1754,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1715,61 +1771,61 @@
       <c r="F4" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="22" t="s">
+      <c r="A6" s="24" t="s">
         <v>73</v>
       </c>
+      <c r="B6" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>74</v>
+      <c r="A7" s="13" t="s">
+        <v>76</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C7" s="16"/>
+        <v>77</v>
+      </c>
+      <c r="C7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="B8" s="11" t="str">
+      <c r="A8" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="13" t="str">
         <f aca="false">B7</f>
         <v>Q3</v>
       </c>
       <c r="C8" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="C10" s="16"/>
+      <c r="A10" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="16"/>
+      <c r="A11" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="16"/>
+      <c r="A12" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1824,7 +1880,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1832,7 +1888,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1846,56 +1902,56 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>85</v>
+      <c r="A7" s="24" t="s">
+        <v>87</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>87</v>
+      <c r="A8" s="13" t="s">
+        <v>89</v>
       </c>
       <c r="B8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" s="16"/>
+      <c r="A9" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>89</v>
+      <c r="A10" s="13" t="s">
+        <v>91</v>
       </c>
       <c r="B10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
+      <c r="A11" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1908,58 +1964,58 @@
       <c r="D16" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="B18" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="C18" s="22" t="s">
+      <c r="A18" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="B18" s="24" t="s">
         <v>96</v>
       </c>
+      <c r="C18" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="n">
+      <c r="A19" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="15" t="n">
+      <c r="B19" s="29"/>
+      <c r="C19" s="17" t="n">
         <v>948</v>
       </c>
-      <c r="D19" s="16"/>
+      <c r="D19" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="13" t="n">
         <v>34</v>
       </c>
-      <c r="B20" s="27"/>
-      <c r="C20" s="15" t="n">
+      <c r="B20" s="29"/>
+      <c r="C20" s="17" t="n">
         <v>2686</v>
       </c>
-      <c r="D20" s="16"/>
+      <c r="D20" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="n">
+      <c r="A21" s="13" t="n">
         <v>73</v>
       </c>
-      <c r="B21" s="27"/>
-      <c r="C21" s="15" t="n">
+      <c r="B21" s="29"/>
+      <c r="C21" s="17" t="n">
         <v>5767</v>
       </c>
-      <c r="D21" s="16"/>
+      <c r="D21" s="18"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="13" t="n">
         <v>150</v>
       </c>
-      <c r="B22" s="27"/>
-      <c r="C22" s="15" t="n">
+      <c r="B22" s="29"/>
+      <c r="C22" s="17" t="n">
         <v>11850</v>
       </c>
-      <c r="D22" s="16"/>
+      <c r="D22" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1998,7 +2054,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2011,269 +2067,269 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" s="22" t="s">
+      <c r="A4" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="B4" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>79</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>189</v>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>329</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>0.07</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>549</v>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>279</v>
+      </c>
+      <c r="E9" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="F4" s="22" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="F9" s="15" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="C5" s="15" t="n">
+      <c r="B11" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>899</v>
+      </c>
+      <c r="E11" s="30" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>94.5</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="C17" s="17" t="n">
         <v>79</v>
       </c>
-      <c r="E5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6" s="15" t="n">
-        <v>189</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="C7" s="15" t="n">
-        <v>329</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>0.07</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="C8" s="15" t="n">
-        <v>549</v>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>50</v>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="C9" s="15" t="n">
-        <v>279</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="C10" s="15" t="n">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="15" t="n">
-        <v>899</v>
-      </c>
-      <c r="E11" s="28" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="C12" s="15" t="n">
-        <v>94.5</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="C13" s="15" t="n">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="C14" s="15" t="n">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="C15" s="15" t="n">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="C16" s="15" t="n">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="C17" s="15" t="n">
-        <v>79</v>
-      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="C18" s="15" t="n">
+      <c r="A18" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C18" s="17" t="n">
         <v>139</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="B22" s="25" t="s">
-        <v>123</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="D22" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="E22" s="25" t="s">
+      <c r="A22" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="27" t="s">
         <v>125</v>
       </c>
+      <c r="C22" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="D22" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="E22" s="27" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="22" t="s">
-        <v>126</v>
-      </c>
-      <c r="B23" s="12" t="n">
+      <c r="A23" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" s="14" t="n">
         <v>612</v>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C23" s="14" t="n">
         <v>548</v>
       </c>
-      <c r="D23" s="12" t="n">
+      <c r="D23" s="14" t="n">
         <v>497</v>
       </c>
-      <c r="E23" s="12" t="n">
+      <c r="E23" s="14" t="n">
         <v>579</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22" t="s">
-        <v>127</v>
-      </c>
-      <c r="B24" s="11" t="n">
+      <c r="A24" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="B24" s="13" t="n">
         <v>184</v>
       </c>
-      <c r="C24" s="11" t="n">
+      <c r="C24" s="13" t="n">
         <v>236</v>
       </c>
-      <c r="D24" s="11" t="n">
+      <c r="D24" s="13" t="n">
         <v>311</v>
       </c>
-      <c r="E24" s="11" t="n">
+      <c r="E24" s="13" t="n">
         <v>402</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Instructies van oefening 1 en 3 verduidelijken
- oefening 1: bij de maandelijkse afbetaling staat nu dezelfde uitleg
  als in de takenlijst (rente door 12, jaren maal 12)
- oefening 3: de codes en aantallen staan al ingevuld, dus vraagt de
  instructie nu om de formules uit rij 7 door te trekken, met uitleg
  hoe dat gaat en wat er dan in de formule verandert
- de taak over de onbestaande code is een onderzoeksvraag geworden,
  want ALS.FOUT zit al in de voorbeeldformule

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wu5SnViXCqMtBpPMNxsmhA
</commit_message>
<xml_diff>
--- a/bestanden/werkbladen-oefeningen-START.xlsx
+++ b/bestanden/werkbladen-oefeningen-START.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="131">
   <si>
     <t xml:space="preserve">Werkbladen — oefeningenbundel</t>
   </si>
@@ -109,7 +109,10 @@
     <t xml:space="preserve">Hoeveel rente kost die lening mij in totaal?</t>
   </si>
   <si>
-    <t xml:space="preserve">Wat als ik maandelijks afbetaal in plaats van jaarlijks? (let op de periodes)</t>
+    <t xml:space="preserve">Wat als ik maandelijks afbetaal in plaats van jaarlijks?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rente en looptijd moeten over dezelfde periode gaan. Deel de rente door 12 en vermenigvuldig het aantal jaren met 12. Vergeet je dat, dan rekent Sheets met 3% per maand.</t>
   </si>
   <si>
     <t xml:space="preserve">Functies die je hier kunt gebruiken (klik voor de uitleg)</t>
@@ -172,7 +175,7 @@
     <t xml:space="preserve">Oefening 3 — Een pc samenstellen met VERT.ZOEKEN</t>
   </si>
   <si>
-    <t xml:space="preserve">Hieronder staat de configuratie van een pc. Vul enkel de artikelcode en het aantal in; de omschrijving en de prijs haal je op uit het blad Gegevens.</t>
+    <t xml:space="preserve">De configuratie van een pc staat al klaar: de artikelcodes en de aantallen zijn ingevuld. In rij 7 staan de formules al als voorbeeld. Trek ze door naar beneden tot en met rij 14, zodat elke rij zijn onderdeel, prijs en totaal ophaalt uit het blad Gegevens. Selecteer daarvoor B7 tot E7, pak het blauwe vierkantje rechtsonder de selectie vast en sleep tot rij 14.</t>
   </si>
   <si>
     <t xml:space="preserve">Code</t>
@@ -196,7 +199,7 @@
     <t xml:space="preserve">CPU-01</t>
   </si>
   <si>
-    <t xml:space="preserve">voorbeeld — kijk hoe het werkt</t>
+    <t xml:space="preserve">voorbeeld: trek deze formules door naar beneden</t>
   </si>
   <si>
     <t xml:space="preserve">MOB-02</t>
@@ -220,7 +223,7 @@
     <t xml:space="preserve">GPU-99</t>
   </si>
   <si>
-    <t xml:space="preserve">deze code bestaat niet — vang de fout netjes op</t>
+    <t xml:space="preserve">deze code bestaat niet, kijk wat er gebeurt</t>
   </si>
   <si>
     <t xml:space="preserve">Totaalprijs van de pc</t>
@@ -431,7 +434,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="&quot;€ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -501,6 +504,14 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF7A8699"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -610,7 +621,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -655,7 +666,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -691,7 +702,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -731,7 +746,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1097,7 +1112,7 @@
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
         <v>12</v>
       </c>
@@ -1111,14 +1126,14 @@
       <c r="D21" s="12"/>
       <c r="E21" s="12"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12"/>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
       <c r="E22" s="12"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12"/>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
@@ -1258,70 +1273,79 @@
       </c>
       <c r="B18" s="18"/>
     </row>
+    <row r="19" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+    </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
-        <v>29</v>
+      <c r="A21" s="21" t="s">
+        <v>30</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
-        <v>31</v>
+      <c r="A22" s="21" t="s">
+        <v>32</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
-        <v>33</v>
+      <c r="A23" s="21" t="s">
+        <v>34</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
-        <v>35</v>
+      <c r="A24" s="21" t="s">
+        <v>36</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
+      <c r="A26" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
+      <c r="A27" s="22"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A4:D5"/>
+    <mergeCell ref="A19:D19"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
@@ -1359,7 +1383,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1367,7 +1391,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1381,7 +1405,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>-200</v>
@@ -1389,7 +1413,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B7" s="15" t="n">
         <v>0.02</v>
@@ -1397,7 +1421,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B8" s="13" t="n">
         <v>5</v>
@@ -1405,53 +1429,53 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="22"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
+      <c r="A13" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22"/>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
+      <c r="A14" s="23"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23"/>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23"/>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1488,7 +1512,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1496,9 +1520,9 @@
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1506,7 +1530,7 @@
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1515,51 +1539,51 @@
       <c r="F4" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="B6" s="24" t="s">
+      <c r="A6" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="B6" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="C6" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="D6" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="E6" s="25" t="s">
         <v>54</v>
       </c>
+      <c r="F6" s="25" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="25" t="str">
+      <c r="A7" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="26" t="str">
         <f aca="false">IFERROR(VLOOKUP($A7,Gegevens!$A$5:$C$18,2,FALSE()),"niet gevonden")</f>
         <v>Processor 6 cores, 4,1 GHz</v>
       </c>
-      <c r="C7" s="26" t="n">
+      <c r="C7" s="27" t="n">
         <f aca="false">IFERROR(VLOOKUP($A7,Gegevens!$A$5:$C$18,3,FALSE()),0)</f>
         <v>189</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="27" t="n">
         <f aca="false">C7*D7</f>
         <v>189</v>
       </c>
-      <c r="F7" s="25" t="s">
-        <v>56</v>
+      <c r="F7" s="26" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="18"/>
@@ -1571,7 +1595,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="18"/>
@@ -1583,7 +1607,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="18"/>
@@ -1595,7 +1619,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="18"/>
@@ -1607,7 +1631,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="18"/>
@@ -1619,7 +1643,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="18"/>
@@ -1631,7 +1655,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="18"/>
@@ -1639,42 +1663,42 @@
         <v>1</v>
       </c>
       <c r="E14" s="18"/>
-      <c r="F14" s="25" t="s">
-        <v>64</v>
+      <c r="F14" s="26" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D16" s="27" t="s">
-        <v>65</v>
+      <c r="D16" s="28" t="s">
+        <v>66</v>
       </c>
       <c r="E16" s="18"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D17" s="27" t="s">
-        <v>66</v>
+      <c r="D17" s="28" t="s">
+        <v>67</v>
       </c>
       <c r="E17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D18" s="27" t="s">
-        <v>67</v>
+      <c r="D18" s="28" t="s">
+        <v>68</v>
       </c>
       <c r="E18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D19" s="27" t="s">
-        <v>68</v>
+      <c r="D19" s="28" t="s">
+        <v>69</v>
       </c>
       <c r="E19" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1744,7 +1768,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1754,7 +1778,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1771,28 +1795,28 @@
       <c r="F4" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="24" t="s">
+      <c r="A6" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="B6" s="25" t="s">
         <v>75</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="13" t="str">
         <f aca="false">B7</f>
@@ -1802,30 +1826,30 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C12" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1880,7 +1904,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1888,7 +1912,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1902,56 +1926,56 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>87</v>
+      <c r="A7" s="25" t="s">
+        <v>88</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
+      <c r="A11" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1964,24 +1988,24 @@
       <c r="D16" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="24" t="s">
-        <v>95</v>
-      </c>
-      <c r="B18" s="24" t="s">
+      <c r="A18" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="B18" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="C18" s="25" t="s">
         <v>98</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="29"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="17" t="n">
         <v>948</v>
       </c>
@@ -1991,7 +2015,7 @@
       <c r="A20" s="13" t="n">
         <v>34</v>
       </c>
-      <c r="B20" s="29"/>
+      <c r="B20" s="30"/>
       <c r="C20" s="17" t="n">
         <v>2686</v>
       </c>
@@ -2001,7 +2025,7 @@
       <c r="A21" s="13" t="n">
         <v>73</v>
       </c>
-      <c r="B21" s="29"/>
+      <c r="B21" s="30"/>
       <c r="C21" s="17" t="n">
         <v>5767</v>
       </c>
@@ -2011,7 +2035,7 @@
       <c r="A22" s="13" t="n">
         <v>150</v>
       </c>
-      <c r="B22" s="29"/>
+      <c r="B22" s="30"/>
       <c r="C22" s="17" t="n">
         <v>11850</v>
       </c>
@@ -2054,7 +2078,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2067,35 +2091,35 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="24" t="s">
+      <c r="A4" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="B4" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="24" t="s">
-        <v>102</v>
-      </c>
-      <c r="F4" s="24" t="s">
-        <v>96</v>
+      <c r="C4" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>79</v>
@@ -2109,10 +2133,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>189</v>
@@ -2126,10 +2150,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>329</v>
@@ -2143,10 +2167,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>549</v>
@@ -2160,10 +2184,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>279</v>
@@ -2177,10 +2201,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>489</v>
@@ -2188,24 +2212,24 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>899</v>
       </c>
-      <c r="E11" s="30" t="s">
-        <v>114</v>
+      <c r="E11" s="31" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>94.5</v>
@@ -2213,10 +2237,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>109</v>
@@ -2224,10 +2248,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>179</v>
@@ -2235,10 +2259,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C15" s="17" t="n">
         <v>89</v>
@@ -2246,10 +2270,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C16" s="17" t="n">
         <v>64</v>
@@ -2257,10 +2281,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C17" s="17" t="n">
         <v>79</v>
@@ -2268,10 +2292,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C18" s="17" t="n">
         <v>139</v>
@@ -2279,29 +2303,29 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="24" t="s">
-        <v>74</v>
-      </c>
-      <c r="B22" s="27" t="s">
-        <v>125</v>
-      </c>
-      <c r="C22" s="27" t="s">
+      <c r="A22" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="28" t="s">
         <v>126</v>
       </c>
-      <c r="D22" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="E22" s="27" t="s">
+      <c r="C22" s="28" t="s">
         <v>127</v>
       </c>
+      <c r="D22" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="E22" s="28" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="24" t="s">
-        <v>128</v>
+      <c r="A23" s="25" t="s">
+        <v>129</v>
       </c>
       <c r="B23" s="14" t="n">
         <v>612</v>
@@ -2317,8 +2341,8 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="24" t="s">
-        <v>129</v>
+      <c r="A24" s="25" t="s">
+        <v>130</v>
       </c>
       <c r="B24" s="13" t="n">
         <v>184</v>

</xml_diff>